<commit_message>
Add ranking regression coverage
Co-authored-by: Chapel-Saint-Auret <202953856+Chapel-Saint-Auret@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/release_format_mismatched_names.xlsx
+++ b/tests/fixtures/release_format_mismatched_names.xlsx
@@ -431,7 +431,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>RPLC - C18 - ACN/H$_2$O - pH 3</t>
+          <t>RPLC - C18 - ACN/H2O - pH 3</t>
         </is>
       </c>
     </row>
@@ -497,7 +497,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>RPLC - Wrong - ACN/H$_2$O - pH 3</t>
+          <t>RPLC - Wrong - ACN/H2O - pH 3</t>
         </is>
       </c>
     </row>
@@ -537,7 +537,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>RPLC - Wrong - ACN/H$_2$O - pH 3</t>
+          <t>RPLC - Wrong - ACN/H2O - pH 3</t>
         </is>
       </c>
     </row>

</xml_diff>